<commit_message>
Document account rules for booking
Customers never have accounts; their details live only on the payment-bearing
appointment or order. Barbers are created by the owner (users + barbers rows
in one form) and sign in to their own /barber area by emailed code only.
Barber access comes from barbers.user_id + is_active, so no schema change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/booking-flows.xlsx
+++ b/docs/booking-flows.xlsx
@@ -16,7 +16,7 @@
     <sheet name="Insert audit" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Features!$A$1:$F$32</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Features!$A$1:$F$35</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Flows!$A$1:$L$51</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="990" uniqueCount="597">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1016" uniqueCount="613">
   <si>
     <t xml:space="preserve">Booking system: flows &amp; features</t>
   </si>
@@ -187,25 +187,25 @@
     <t xml:space="preserve">FND-02</t>
   </si>
   <si>
-    <t xml:space="preserve">Barber role &amp; login</t>
+    <t xml:space="preserve">Barber sign-in (email code only)</t>
   </si>
   <si>
     <t xml:space="preserve">Barber</t>
   </si>
   <si>
-    <t xml:space="preserve">Barber opens /admin/login</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Barber enters email -&gt; same email-OTP flow the owner uses.
-2. The admin lookup becomes a staff lookup: role admin, OR a user linked from an active barbers row.
-3. Session carries role + linked barber_id.
-4. Admin layout shows only the barber menu for role barber.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">users, barbers, sessions, otp_codes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A barber login with no linked barbers row sees 'ask the owner to link your profile'. Role is re-checked at code verification, as it is for admins today.</t>
+    <t xml:space="preserve">Barber opens /barber/login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Barber enters their email -&gt; the same 6-digit emailed code flow as /admin/login. No passwords anywhere.
+2. A code is only sent if the email belongs to a user linked from an ACTIVE barbers row; the page answers the same either way.
+3. Verify -&gt; re-check the link is still active -&gt; database session cookie (same sessions table as the owner).
+4. Lands in the barber's own area, /barber, scoped to their barbers row.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">users, barbers, otp_codes, sessions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barber access comes from barbers.user_id + is_active, not users.role. Deactivating a barber stops new codes and is re-checked on every request, so open sessions stop working too. An owner who is also a barber uses one session for both /admin and /barber.</t>
   </si>
   <si>
     <t xml:space="preserve">FND-03</t>
@@ -251,21 +251,22 @@
     <t xml:space="preserve">OWN-02</t>
   </si>
   <si>
-    <t xml:space="preserve">Create barber &amp; grant login</t>
+    <t xml:space="preserve">Create a barber (owner's form)</t>
   </si>
   <si>
     <t xml:space="preserve">New barber joins</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Create barbers row: name, slug, phone (required), photo, bio, booking fee, buffer.
-2. Grant login: create or promote a users row with role barber and link barbers.user_id.
-3. Set their terms (OWN-03).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">barbers, users, barber_terms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phone is required: customers see it on every confirmation. A barber can exist without a login; the owner then manages them.</t>
+    <t xml:space="preserve">1. Owner fills one form: login email, name, phone, photo, bio, booking fee, buffer.
+2. ONE transaction: insert the users row (or reuse the existing user with that email, e.g. the owner themselves) + the barbers row linked by user_id.
+3. Set their terms (OWN-03).
+4. The barber can now sign in at /barber/login with an emailed code.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">users, barbers, barber_terms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No self-signup and no passwords: only the owner creates barbers. Phone is required (customers see it). Login email must be unique across users.</t>
   </si>
   <si>
     <t xml:space="preserve">OWN-03</t>
@@ -307,7 +308,7 @@
   </si>
   <si>
     <t xml:space="preserve">1. Set is_active = false; hidden from online booking.
-2. Revoke login (unlink barbers.user_id, sessions deleted).
+2. Access ends immediately: sign-in and every /barber request check is_active; their sessions are deleted too.
 3. Owner sees their future appointments to reassign or cancel by phone.</t>
   </si>
   <si>
@@ -1388,6 +1389,27 @@
     <t xml:space="preserve">BAR-01, BAR-03</t>
   </si>
   <si>
+    <t xml:space="preserve">Customers never have accounts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Their name, phone and email live only on the appointment or order that carries their payment; everything reaches them by email.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CUS-02, CUS-04, NTF-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barbers sign in by email code only, to their own area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same 6-digit emailed code as the owner, no passwords; /barber shows only the signed-in barber's data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only the owner creates barbers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One form creates the login and the barber profile together; no self-signup.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Owner can also be a barber</t>
   </si>
   <si>
@@ -1592,6 +1614,18 @@
     <t xml:space="preserve">Who took it = in_store_sales.barber_id.</t>
   </si>
   <si>
+    <t xml:space="preserve">otp_codes, sessions (unchanged)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emailed-code sign-in and sessions.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No changes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Serve both /admin and /barber sign-in.</t>
+  </si>
+  <si>
     <t xml:space="preserve">users (unchanged)</t>
   </si>
   <si>
@@ -1607,6 +1641,24 @@
     <t xml:space="preserve">Action</t>
   </si>
   <si>
+    <t xml:space="preserve">Sign in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/admin, emailed code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/barber, emailed code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No account</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create barbers and their logins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes</t>
+  </si>
+  <si>
     <t xml:space="preserve">Products, prices, stock, settings</t>
   </si>
   <si>
@@ -1626,9 +1678,6 @@
   </si>
   <si>
     <t xml:space="preserve">Rent charges: confirm / waive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes</t>
   </si>
   <si>
     <t xml:space="preserve">Payouts, cash hand-ins, adjustments</t>
@@ -2852,15 +2901,15 @@
         <v>29</v>
       </c>
       <c r="B27" s="8" t="n">
-        <f aca="false">COUNTA(Features!$B$2:$B$32)</f>
-        <v>31</v>
+        <f aca="false">COUNTA(Features!$B$2:$B$35)</f>
+        <v>34</v>
       </c>
       <c r="C27" s="8" t="n">
-        <f aca="false">COUNTIF(Features!$E$2:$E$32,"Done")</f>
+        <f aca="false">COUNTIF(Features!$E$2:$E$35,"Done")</f>
         <v>0</v>
       </c>
       <c r="D27" s="8" t="n">
-        <f aca="false">COUNTIF(Features!$E$2:$E$32,"In progress")</f>
+        <f aca="false">COUNTIF(Features!$E$2:$E$35,"In progress")</f>
         <v>0</v>
       </c>
       <c r="E27" s="9" t="n">
@@ -2975,7 +3024,7 @@
       </c>
       <c r="L2" s="12"/>
     </row>
-    <row r="3" customFormat="false" ht="69" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
         <v>50</v>
       </c>
@@ -3083,7 +3132,7 @@
       </c>
       <c r="L5" s="12"/>
     </row>
-    <row r="6" customFormat="false" ht="69" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="81.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
         <v>69</v>
       </c>
@@ -3155,7 +3204,7 @@
       </c>
       <c r="L7" s="12"/>
     </row>
-    <row r="8" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
         <v>83</v>
       </c>
@@ -4774,7 +4823,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -5327,7 +5376,7 @@
       </c>
       <c r="F30" s="12"/>
     </row>
-    <row r="31" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="n">
         <v>30</v>
       </c>
@@ -5338,7 +5387,7 @@
         <v>425</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>90</v>
+        <v>426</v>
       </c>
       <c r="E31" s="12" t="s">
         <v>8</v>
@@ -5350,22 +5399,76 @@
         <v>31</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="D32" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="E32" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F32" s="12"/>
+    </row>
+    <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>429</v>
+      </c>
+      <c r="C33" s="11" t="s">
+        <v>430</v>
+      </c>
+      <c r="D33" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="E33" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" s="12"/>
+    </row>
+    <row r="34" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="11" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>431</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="D34" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="E34" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F34" s="12"/>
+    </row>
+    <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="11" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>433</v>
+      </c>
+      <c r="C35" s="11" t="s">
+        <v>434</v>
+      </c>
+      <c r="D35" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="E32" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="F32" s="12"/>
+      <c r="E35" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F35" s="12"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F32"/>
-  <conditionalFormatting sqref="E2:E32">
+  <autoFilter ref="A1:F35"/>
+  <conditionalFormatting sqref="E2:E35">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>$E2="Done"</formula>
     </cfRule>
@@ -5377,7 +5480,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" error="Pick a status from the list" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E32" type="list">
+    <dataValidation allowBlank="false" error="Pick a status from the list" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E35" type="list">
       <formula1>"To do,In progress,Done,Blocked"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -5398,7 +5501,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -5410,22 +5513,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>428</v>
+        <v>435</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>430</v>
+        <v>437</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>431</v>
+        <v>438</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5433,19 +5536,19 @@
         <v>67</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="C2" s="11" t="s">
         <v>64</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>435</v>
+        <v>442</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5453,19 +5556,19 @@
         <v>100</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>438</v>
+        <v>445</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>439</v>
+        <v>446</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>440</v>
+        <v>447</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5473,19 +5576,19 @@
         <v>105</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>442</v>
+        <v>449</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>52</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>443</v>
+        <v>450</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>444</v>
+        <v>451</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>445</v>
+        <v>452</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5493,19 +5596,19 @@
         <v>116</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>442</v>
+        <v>449</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>52</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>446</v>
+        <v>453</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>447</v>
+        <v>454</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5513,19 +5616,19 @@
         <v>81</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>449</v>
+        <v>456</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>64</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>450</v>
+        <v>457</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>451</v>
+        <v>458</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>452</v>
+        <v>459</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5533,19 +5636,19 @@
         <v>304</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>449</v>
+        <v>456</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>453</v>
+        <v>460</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>455</v>
+        <v>462</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>456</v>
+        <v>463</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5553,79 +5656,79 @@
         <v>338</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>459</v>
+        <v>466</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>460</v>
+        <v>467</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>461</v>
+        <v>468</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>52</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>463</v>
+        <v>470</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>464</v>
+        <v>471</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>465</v>
+        <v>472</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>466</v>
+        <v>473</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>131</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>467</v>
+        <v>474</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>468</v>
+        <v>475</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>469</v>
+        <v>476</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>470</v>
+        <v>477</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>472</v>
+        <v>479</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>473</v>
+        <v>480</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>474</v>
+        <v>481</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5636,96 +5739,116 @@
         <v>24</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>475</v>
+        <v>482</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>476</v>
+        <v>483</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>477</v>
+        <v>484</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>478</v>
+        <v>485</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>479</v>
+        <v>486</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>52</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>480</v>
+        <v>487</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>481</v>
+        <v>488</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>482</v>
+        <v>489</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>483</v>
+        <v>490</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>484</v>
+        <v>491</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>49</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>485</v>
+        <v>492</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>486</v>
+        <v>493</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>487</v>
+        <v>494</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>488</v>
+        <v>495</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>484</v>
+        <v>491</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>49</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>489</v>
+        <v>496</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>490</v>
+        <v>497</v>
       </c>
       <c r="F15" s="11" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
+        <v>499</v>
+      </c>
+      <c r="B16" s="11" t="s">
         <v>491</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
-        <v>492</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>484</v>
-      </c>
       <c r="C16" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>500</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>501</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="s">
+        <v>503</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>491</v>
+      </c>
+      <c r="C17" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="D16" s="11" t="s">
-        <v>493</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>494</v>
-      </c>
-      <c r="F16" s="11" t="s">
-        <v>495</v>
+      <c r="D17" s="11" t="s">
+        <v>504</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>505</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>506</v>
       </c>
     </row>
   </sheetData>
@@ -5744,7 +5867,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -5755,7 +5878,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>496</v>
+        <v>507</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>64</v>
@@ -5769,41 +5892,41 @@
     </row>
     <row r="2" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>497</v>
+        <v>508</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>498</v>
+        <v>509</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>49</v>
+        <v>510</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>49</v>
+        <v>511</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>499</v>
+        <v>512</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>498</v>
+        <v>513</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>500</v>
+        <v>49</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>500</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>501</v>
+        <v>514</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>498</v>
+        <v>515</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>502</v>
+        <v>49</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>49</v>
@@ -5811,27 +5934,27 @@
     </row>
     <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>503</v>
+        <v>516</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>504</v>
+        <v>515</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>502</v>
+        <v>517</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>49</v>
+        <v>517</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>505</v>
+        <v>518</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>504</v>
+        <v>515</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>502</v>
+        <v>519</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>49</v>
@@ -5839,13 +5962,13 @@
     </row>
     <row r="7" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>506</v>
+        <v>520</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>508</v>
+        <v>519</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>49</v>
@@ -5853,27 +5976,27 @@
     </row>
     <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>509</v>
+        <v>521</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>508</v>
+        <v>519</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>510</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>511</v>
+        <v>522</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>507</v>
+        <v>523</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>508</v>
+        <v>524</v>
       </c>
       <c r="D9" s="11" t="s">
         <v>49</v>
@@ -5881,27 +6004,27 @@
     </row>
     <row r="10" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>512</v>
+        <v>525</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>49</v>
+        <v>523</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>49</v>
+        <v>524</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>504</v>
+        <v>526</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>513</v>
+        <v>527</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>504</v>
+        <v>523</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>514</v>
+        <v>524</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>49</v>
@@ -5909,27 +6032,27 @@
     </row>
     <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>515</v>
+        <v>528</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>504</v>
+        <v>49</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>514</v>
+        <v>49</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>517</v>
+        <v>529</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>504</v>
+        <v>513</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>514</v>
+        <v>530</v>
       </c>
       <c r="D13" s="11" t="s">
         <v>49</v>
@@ -5937,27 +6060,27 @@
     </row>
     <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>518</v>
+        <v>531</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>504</v>
+        <v>513</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>519</v>
+        <v>530</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>520</v>
+        <v>532</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>521</v>
+        <v>533</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>504</v>
+        <v>513</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>522</v>
+        <v>530</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>49</v>
@@ -5965,15 +6088,43 @@
     </row>
     <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>523</v>
+        <v>534</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>524</v>
+        <v>513</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>514</v>
+        <v>535</v>
       </c>
       <c r="D16" s="11" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11" t="s">
+        <v>537</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>513</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>538</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
+        <v>539</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>540</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>530</v>
+      </c>
+      <c r="D18" s="11" t="s">
         <v>49</v>
       </c>
     </row>
@@ -6005,90 +6156,90 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>525</v>
+        <v>541</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>526</v>
+        <v>542</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>527</v>
+        <v>543</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>528</v>
+        <v>544</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>529</v>
+        <v>545</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>530</v>
+        <v>546</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>531</v>
+        <v>547</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>532</v>
+        <v>548</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>533</v>
+        <v>549</v>
       </c>
       <c r="D2" s="11" t="s">
         <v>49</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>534</v>
+        <v>550</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>535</v>
+        <v>551</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>536</v>
+        <v>552</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>537</v>
+        <v>553</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>533</v>
+        <v>549</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>538</v>
+        <v>554</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>539</v>
+        <v>555</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>540</v>
+        <v>556</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>541</v>
+        <v>557</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>542</v>
+        <v>558</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>543</v>
+        <v>559</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>504</v>
+        <v>513</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>544</v>
+        <v>560</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>545</v>
+        <v>561</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>546</v>
+        <v>562</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>547</v>
+        <v>563</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>131</v>
@@ -6097,155 +6248,155 @@
         <v>49</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>548</v>
+        <v>564</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>549</v>
+        <v>565</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>550</v>
+        <v>566</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>551</v>
+        <v>567</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>533</v>
+        <v>549</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>552</v>
+        <v>568</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>554</v>
+        <v>570</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>555</v>
+        <v>571</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>556</v>
+        <v>572</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>557</v>
+        <v>573</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>552</v>
+        <v>568</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>558</v>
+        <v>574</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>559</v>
+        <v>575</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>560</v>
+        <v>576</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>561</v>
+        <v>577</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>557</v>
+        <v>573</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>552</v>
+        <v>568</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>562</v>
+        <v>578</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>563</v>
+        <v>579</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>564</v>
+        <v>580</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>565</v>
+        <v>581</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>557</v>
+        <v>573</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>566</v>
+        <v>582</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>544</v>
+        <v>560</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>567</v>
+        <v>583</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>568</v>
+        <v>584</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>532</v>
+        <v>548</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>557</v>
+        <v>573</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>49</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>534</v>
+        <v>550</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>569</v>
+        <v>585</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>570</v>
+        <v>586</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>571</v>
+        <v>587</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>557</v>
+        <v>573</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>572</v>
+        <v>588</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>544</v>
+        <v>560</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>573</v>
+        <v>589</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>574</v>
+        <v>590</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>575</v>
+        <v>591</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>576</v>
+        <v>592</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>552</v>
+        <v>568</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>562</v>
+        <v>578</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>577</v>
+        <v>593</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>578</v>
+        <v>594</v>
       </c>
       <c r="B13" s="11" t="s">
         <v>304</v>
@@ -6254,18 +6405,18 @@
         <v>131</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>579</v>
+        <v>595</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>562</v>
+        <v>578</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>580</v>
+        <v>596</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>581</v>
+        <v>597</v>
       </c>
       <c r="B14" s="11" t="s">
         <v>254</v>
@@ -6274,41 +6425,41 @@
         <v>131</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>504</v>
+        <v>513</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>544</v>
+        <v>560</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>582</v>
+        <v>598</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>583</v>
+        <v>599</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>584</v>
+        <v>600</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>585</v>
+        <v>601</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>566</v>
+        <v>582</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>544</v>
+        <v>560</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>586</v>
+        <v>602</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>587</v>
+        <v>603</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>588</v>
+        <v>604</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>131</v>
@@ -6317,7 +6468,7 @@
         <v>49</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>534</v>
+        <v>550</v>
       </c>
       <c r="F16" s="11" t="s">
         <v>49</v>
@@ -6325,42 +6476,42 @@
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>589</v>
+        <v>605</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>590</v>
+        <v>606</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>591</v>
+        <v>607</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>552</v>
+        <v>568</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>562</v>
+        <v>578</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>592</v>
+        <v>608</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>593</v>
+        <v>609</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>594</v>
+        <v>610</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>533</v>
+        <v>549</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>552</v>
+        <v>568</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>595</v>
+        <v>611</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>596</v>
+        <v>612</v>
       </c>
     </row>
   </sheetData>

</xml_diff>